<commit_message>
fix(hardware): added routing for flow signal and added pull-up resistors for easy bootloader flash
</commit_message>
<xml_diff>
--- a/hardware/ThermalFlowMeter-BoM.xlsx
+++ b/hardware/ThermalFlowMeter-BoM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="224">
   <si>
     <t>No.</t>
   </si>
@@ -73,7 +73,7 @@
     <t>LCSC</t>
   </si>
   <si>
-    <t>0.0037</t>
+    <t>0.0006</t>
   </si>
   <si>
     <t>2</t>
@@ -94,7 +94,7 @@
     <t>C1713</t>
   </si>
   <si>
-    <t>0.0077</t>
+    <t>0.0013</t>
   </si>
   <si>
     <t>3</t>
@@ -112,7 +112,7 @@
     <t>C215803</t>
   </si>
   <si>
-    <t>0.009</t>
+    <t>0.0014</t>
   </si>
   <si>
     <t>4</t>
@@ -130,7 +130,7 @@
     <t>C1779</t>
   </si>
   <si>
-    <t>0.0104</t>
+    <t>0.0018</t>
   </si>
   <si>
     <t>5</t>
@@ -154,7 +154,7 @@
     <t>C694469</t>
   </si>
   <si>
-    <t>0.2271</t>
+    <t>0.0505</t>
   </si>
   <si>
     <t>6</t>
@@ -172,7 +172,7 @@
     <t>C5674</t>
   </si>
   <si>
-    <t>0.0108</t>
+    <t>0.0016</t>
   </si>
   <si>
     <t>7</t>
@@ -196,9 +196,6 @@
     <t>C2986110</t>
   </si>
   <si>
-    <t>0.0094</t>
-  </si>
-  <si>
     <t>8</t>
   </si>
   <si>
@@ -217,7 +214,7 @@
     <t>C210839</t>
   </si>
   <si>
-    <t>0.125</t>
+    <t>0.0191</t>
   </si>
   <si>
     <t>9</t>
@@ -241,7 +238,7 @@
     <t>C492265</t>
   </si>
   <si>
-    <t>0.0387</t>
+    <t>0.0054</t>
   </si>
   <si>
     <t>10</t>
@@ -262,7 +259,7 @@
     <t>C965812</t>
   </si>
   <si>
-    <t>0.0058</t>
+    <t>0.0008</t>
   </si>
   <si>
     <t>11</t>
@@ -283,7 +280,7 @@
     <t>C5290371</t>
   </si>
   <si>
-    <t>0.246</t>
+    <t>0.0502</t>
   </si>
   <si>
     <t>12</t>
@@ -301,7 +298,7 @@
     <t>C5290369</t>
   </si>
   <si>
-    <t>0.1781</t>
+    <t>0.0355</t>
   </si>
   <si>
     <t>13</t>
@@ -322,7 +319,7 @@
     <t>C65114</t>
   </si>
   <si>
-    <t>0.0296</t>
+    <t>0.0043</t>
   </si>
   <si>
     <t>14</t>
@@ -343,7 +340,7 @@
     <t>C319148</t>
   </si>
   <si>
-    <t>0.2501</t>
+    <t>0.0309</t>
   </si>
   <si>
     <t>15</t>
@@ -373,7 +370,7 @@
     <t>10kΩ</t>
   </si>
   <si>
-    <t>R3,R4,R9</t>
+    <t>R3,R4,R9,R18,R19,R20</t>
   </si>
   <si>
     <t>0805W8F1002T5E</t>
@@ -385,7 +382,7 @@
     <t>C17414</t>
   </si>
   <si>
-    <t>0.0017</t>
+    <t>0.0003</t>
   </si>
   <si>
     <t>17</t>
@@ -421,9 +418,6 @@
     <t>C269736</t>
   </si>
   <si>
-    <t>0.0038</t>
-  </si>
-  <si>
     <t>19</t>
   </si>
   <si>
@@ -439,9 +433,6 @@
     <t>C17561</t>
   </si>
   <si>
-    <t>0.0019</t>
-  </si>
-  <si>
     <t>20</t>
   </si>
   <si>
@@ -457,7 +448,7 @@
     <t>C840634</t>
   </si>
   <si>
-    <t>0.1527</t>
+    <t>0.0278</t>
   </si>
   <si>
     <t>21</t>
@@ -478,7 +469,7 @@
     <t>C101915</t>
   </si>
   <si>
-    <t>0.0028</t>
+    <t>0.0004</t>
   </si>
   <si>
     <t>22</t>
@@ -499,9 +490,6 @@
     <t>C228750</t>
   </si>
   <si>
-    <t>0.0039</t>
-  </si>
-  <si>
     <t>23</t>
   </si>
   <si>
@@ -517,9 +505,6 @@
     <t>C17873</t>
   </si>
   <si>
-    <t>0.0018</t>
-  </si>
-  <si>
     <t>24</t>
   </si>
   <si>
@@ -535,9 +520,6 @@
     <t>C204311</t>
   </si>
   <si>
-    <t>0.0103</t>
-  </si>
-  <si>
     <t>25</t>
   </si>
   <si>
@@ -553,7 +535,7 @@
     <t>C318938</t>
   </si>
   <si>
-    <t>0.0398</t>
+    <t>0.0057</t>
   </si>
   <si>
     <t>26</t>
@@ -574,7 +556,7 @@
     <t>C5299505</t>
   </si>
   <si>
-    <t>0.1998</t>
+    <t>0.0341</t>
   </si>
   <si>
     <t>27</t>
@@ -595,7 +577,7 @@
     <t>C118474</t>
   </si>
   <si>
-    <t>2.733</t>
+    <t>0.4788</t>
   </si>
   <si>
     <t>28</t>
@@ -616,7 +598,7 @@
     <t>C481365</t>
   </si>
   <si>
-    <t>1.6875</t>
+    <t>0.2769</t>
   </si>
   <si>
     <t>29</t>
@@ -634,7 +616,7 @@
     <t>C112161</t>
   </si>
   <si>
-    <t>5.244</t>
+    <t>0.7507</t>
   </si>
   <si>
     <t>30</t>
@@ -655,7 +637,7 @@
     <t>C524782</t>
   </si>
   <si>
-    <t>0.4185</t>
+    <t>0.072</t>
   </si>
   <si>
     <t>31</t>
@@ -676,7 +658,7 @@
     <t>C5120765</t>
   </si>
   <si>
-    <t>0.0368</t>
+    <t>0.005</t>
   </si>
   <si>
     <t>32</t>
@@ -700,7 +682,7 @@
     <t>C341525</t>
   </si>
   <si>
-    <t>0.2063</t>
+    <t>0.0323</t>
   </si>
 </sst>
 </file>
@@ -1381,7 +1363,7 @@
         <v>19</v>
       </c>
       <c r="K8" t="s">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="L8" t="s">
         <v>55</v>
@@ -1389,952 +1371,952 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" t="s">
         <v>63</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>64</v>
-      </c>
-      <c r="E9" t="s">
-        <v>65</v>
       </c>
       <c r="F9" t="s">
         <v>58</v>
       </c>
       <c r="G9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H9" t="s">
+        <v>65</v>
+      </c>
+      <c r="I9" t="s">
         <v>66</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K9" t="s">
         <v>67</v>
       </c>
-      <c r="J9" t="s">
-        <v>19</v>
-      </c>
-      <c r="K9" t="s">
-        <v>68</v>
-      </c>
       <c r="L9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
       <c r="C10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D10" t="s">
         <v>70</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>71</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" t="s">
         <v>72</v>
       </c>
-      <c r="F10" t="s">
-        <v>70</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>73</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>74</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
+        <v>19</v>
+      </c>
+      <c r="K10" t="s">
         <v>75</v>
       </c>
-      <c r="J10" t="s">
-        <v>19</v>
-      </c>
-      <c r="K10" t="s">
-        <v>76</v>
-      </c>
       <c r="L10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B11">
         <v>2</v>
       </c>
       <c r="C11" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" t="s">
         <v>78</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>79</v>
-      </c>
-      <c r="E11" t="s">
-        <v>80</v>
       </c>
       <c r="F11" t="s">
         <v>58</v>
       </c>
       <c r="G11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H11" t="s">
+        <v>80</v>
+      </c>
+      <c r="I11" t="s">
         <v>81</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K11" t="s">
         <v>82</v>
       </c>
-      <c r="J11" t="s">
-        <v>19</v>
-      </c>
-      <c r="K11" t="s">
-        <v>83</v>
-      </c>
       <c r="L11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
       <c r="C12" t="s">
+        <v>84</v>
+      </c>
+      <c r="D12" t="s">
         <v>85</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>86</v>
-      </c>
-      <c r="E12" t="s">
-        <v>87</v>
       </c>
       <c r="F12" t="s">
         <v>58</v>
       </c>
       <c r="G12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H12" t="s">
+        <v>87</v>
+      </c>
+      <c r="I12" t="s">
         <v>88</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
+        <v>19</v>
+      </c>
+      <c r="K12" t="s">
         <v>89</v>
       </c>
-      <c r="J12" t="s">
-        <v>19</v>
-      </c>
-      <c r="K12" t="s">
-        <v>90</v>
-      </c>
       <c r="L12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D13" t="s">
         <v>92</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>93</v>
-      </c>
-      <c r="E13" t="s">
-        <v>94</v>
       </c>
       <c r="F13" t="s">
         <v>58</v>
       </c>
       <c r="G13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I13" t="s">
+        <v>94</v>
+      </c>
+      <c r="J13" t="s">
+        <v>19</v>
+      </c>
+      <c r="K13" t="s">
         <v>95</v>
       </c>
-      <c r="J13" t="s">
-        <v>19</v>
-      </c>
-      <c r="K13" t="s">
-        <v>96</v>
-      </c>
       <c r="L13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
+        <v>97</v>
+      </c>
+      <c r="D14" t="s">
         <v>98</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>99</v>
-      </c>
-      <c r="E14" t="s">
-        <v>100</v>
       </c>
       <c r="F14" t="s">
         <v>58</v>
       </c>
       <c r="G14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H14" t="s">
+        <v>100</v>
+      </c>
+      <c r="I14" t="s">
         <v>101</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
+        <v>19</v>
+      </c>
+      <c r="K14" t="s">
         <v>102</v>
       </c>
-      <c r="J14" t="s">
-        <v>19</v>
-      </c>
-      <c r="K14" t="s">
-        <v>103</v>
-      </c>
       <c r="L14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
+        <v>104</v>
+      </c>
+      <c r="D15" t="s">
         <v>105</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>106</v>
-      </c>
-      <c r="E15" t="s">
-        <v>107</v>
       </c>
       <c r="F15" t="s">
         <v>58</v>
       </c>
       <c r="G15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H15" t="s">
+        <v>107</v>
+      </c>
+      <c r="I15" t="s">
         <v>108</v>
       </c>
-      <c r="I15" t="s">
+      <c r="J15" t="s">
+        <v>19</v>
+      </c>
+      <c r="K15" t="s">
         <v>109</v>
       </c>
-      <c r="J15" t="s">
-        <v>19</v>
-      </c>
-      <c r="K15" t="s">
-        <v>110</v>
-      </c>
       <c r="L15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B16">
         <v>2</v>
       </c>
       <c r="C16" t="s">
+        <v>111</v>
+      </c>
+      <c r="D16" t="s">
         <v>112</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>113</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
+        <v>111</v>
+      </c>
+      <c r="G16" t="s">
         <v>114</v>
       </c>
-      <c r="F16" t="s">
-        <v>112</v>
-      </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>115</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>116</v>
       </c>
-      <c r="I16" t="s">
-        <v>117</v>
-      </c>
       <c r="J16" t="s">
         <v>19</v>
       </c>
       <c r="K16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>117</v>
+      </c>
+      <c r="B17">
+        <v>6</v>
+      </c>
+      <c r="C17" t="s">
         <v>118</v>
       </c>
-      <c r="B17">
-        <v>3</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>119</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
+        <v>113</v>
+      </c>
+      <c r="F17" t="s">
+        <v>118</v>
+      </c>
+      <c r="G17" t="s">
         <v>120</v>
       </c>
-      <c r="E17" t="s">
-        <v>114</v>
-      </c>
-      <c r="F17" t="s">
-        <v>119</v>
-      </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>121</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>122</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K17" t="s">
         <v>123</v>
       </c>
-      <c r="J17" t="s">
-        <v>19</v>
-      </c>
-      <c r="K17" t="s">
-        <v>124</v>
-      </c>
       <c r="L17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B18">
         <v>2</v>
       </c>
       <c r="C18" t="s">
+        <v>125</v>
+      </c>
+      <c r="D18" t="s">
         <v>126</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
+        <v>113</v>
+      </c>
+      <c r="F18" t="s">
+        <v>125</v>
+      </c>
+      <c r="G18" t="s">
         <v>127</v>
       </c>
-      <c r="E18" t="s">
-        <v>114</v>
-      </c>
-      <c r="F18" t="s">
-        <v>126</v>
-      </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
+        <v>121</v>
+      </c>
+      <c r="I18" t="s">
         <v>128</v>
       </c>
-      <c r="H18" t="s">
-        <v>122</v>
-      </c>
-      <c r="I18" t="s">
-        <v>129</v>
-      </c>
       <c r="J18" t="s">
         <v>19</v>
       </c>
       <c r="K18" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="L18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B19">
         <v>2</v>
       </c>
       <c r="C19" t="s">
+        <v>130</v>
+      </c>
+      <c r="D19" t="s">
         <v>131</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
+        <v>113</v>
+      </c>
+      <c r="F19" t="s">
+        <v>130</v>
+      </c>
+      <c r="G19" t="s">
         <v>132</v>
       </c>
-      <c r="E19" t="s">
-        <v>114</v>
-      </c>
-      <c r="F19" t="s">
-        <v>131</v>
-      </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>133</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>134</v>
       </c>
-      <c r="I19" t="s">
-        <v>135</v>
-      </c>
       <c r="J19" t="s">
         <v>19</v>
       </c>
       <c r="K19" t="s">
-        <v>136</v>
+        <v>20</v>
       </c>
       <c r="L19" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B20">
         <v>2</v>
       </c>
       <c r="C20" t="s">
+        <v>136</v>
+      </c>
+      <c r="D20" t="s">
+        <v>137</v>
+      </c>
+      <c r="E20" t="s">
+        <v>113</v>
+      </c>
+      <c r="F20" t="s">
+        <v>136</v>
+      </c>
+      <c r="G20" t="s">
         <v>138</v>
       </c>
-      <c r="D20" t="s">
+      <c r="H20" t="s">
+        <v>121</v>
+      </c>
+      <c r="I20" t="s">
         <v>139</v>
       </c>
-      <c r="E20" t="s">
-        <v>114</v>
-      </c>
-      <c r="F20" t="s">
-        <v>138</v>
-      </c>
-      <c r="G20" t="s">
-        <v>140</v>
-      </c>
-      <c r="H20" t="s">
-        <v>122</v>
-      </c>
-      <c r="I20" t="s">
-        <v>141</v>
-      </c>
       <c r="J20" t="s">
         <v>19</v>
       </c>
       <c r="K20" t="s">
-        <v>142</v>
+        <v>123</v>
       </c>
       <c r="L20" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B21">
         <v>2</v>
       </c>
       <c r="C21" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D21" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E21" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F21" t="s">
         <v>58</v>
       </c>
       <c r="G21" t="s">
+        <v>141</v>
+      </c>
+      <c r="H21" t="s">
+        <v>65</v>
+      </c>
+      <c r="I21" t="s">
         <v>144</v>
       </c>
-      <c r="H21" t="s">
-        <v>66</v>
-      </c>
-      <c r="I21" t="s">
-        <v>147</v>
-      </c>
       <c r="J21" t="s">
         <v>19</v>
       </c>
       <c r="K21" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="L21" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
       <c r="C22" t="s">
+        <v>147</v>
+      </c>
+      <c r="D22" t="s">
+        <v>148</v>
+      </c>
+      <c r="E22" t="s">
+        <v>113</v>
+      </c>
+      <c r="F22" t="s">
+        <v>147</v>
+      </c>
+      <c r="G22" t="s">
+        <v>149</v>
+      </c>
+      <c r="H22" t="s">
         <v>150</v>
       </c>
-      <c r="D22" t="s">
+      <c r="I22" t="s">
         <v>151</v>
       </c>
-      <c r="E22" t="s">
-        <v>114</v>
-      </c>
-      <c r="F22" t="s">
-        <v>150</v>
-      </c>
-      <c r="G22" t="s">
+      <c r="J22" t="s">
+        <v>19</v>
+      </c>
+      <c r="K22" t="s">
         <v>152</v>
       </c>
-      <c r="H22" t="s">
-        <v>153</v>
-      </c>
-      <c r="I22" t="s">
-        <v>154</v>
-      </c>
-      <c r="J22" t="s">
-        <v>19</v>
-      </c>
-      <c r="K22" t="s">
-        <v>155</v>
-      </c>
       <c r="L22" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
       <c r="C23" t="s">
+        <v>154</v>
+      </c>
+      <c r="D23" t="s">
+        <v>155</v>
+      </c>
+      <c r="E23" t="s">
+        <v>113</v>
+      </c>
+      <c r="F23" t="s">
+        <v>154</v>
+      </c>
+      <c r="G23" t="s">
+        <v>156</v>
+      </c>
+      <c r="H23" t="s">
         <v>157</v>
       </c>
-      <c r="D23" t="s">
+      <c r="I23" t="s">
         <v>158</v>
       </c>
-      <c r="E23" t="s">
-        <v>114</v>
-      </c>
-      <c r="F23" t="s">
-        <v>157</v>
-      </c>
-      <c r="G23" t="s">
-        <v>159</v>
-      </c>
-      <c r="H23" t="s">
-        <v>160</v>
-      </c>
-      <c r="I23" t="s">
-        <v>161</v>
-      </c>
       <c r="J23" t="s">
         <v>19</v>
       </c>
       <c r="K23" t="s">
-        <v>162</v>
+        <v>20</v>
       </c>
       <c r="L23" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B24">
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="D24" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="E24" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F24" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="G24" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="H24" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="I24" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="J24" t="s">
         <v>19</v>
       </c>
       <c r="K24" t="s">
-        <v>168</v>
+        <v>123</v>
       </c>
       <c r="L24" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="B25">
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="D25" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E25" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F25" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="G25" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="H25" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I25" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="J25" t="s">
         <v>19</v>
       </c>
       <c r="K25" t="s">
-        <v>174</v>
+        <v>53</v>
       </c>
       <c r="L25" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="B26">
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="D26" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="E26" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="F26" t="s">
         <v>58</v>
       </c>
       <c r="G26" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="H26" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I26" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="J26" t="s">
         <v>19</v>
       </c>
       <c r="K26" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="L26" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="B27">
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="D27" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="E27" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="F27" t="s">
         <v>58</v>
       </c>
       <c r="G27" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="H27" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="I27" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="J27" t="s">
         <v>19</v>
       </c>
       <c r="K27" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="L27" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B28">
         <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="D28" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E28" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="F28" t="s">
         <v>58</v>
       </c>
       <c r="G28" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="H28" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="I28" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="J28" t="s">
         <v>19</v>
       </c>
       <c r="K28" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="L28" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="B29">
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="D29" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="E29" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="F29" t="s">
         <v>58</v>
       </c>
       <c r="G29" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="H29" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="I29" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="J29" t="s">
         <v>19</v>
       </c>
       <c r="K29" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="L29" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="B30">
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="D30" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="E30" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="F30" t="s">
         <v>58</v>
       </c>
       <c r="G30" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="H30" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="I30" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="J30" t="s">
         <v>19</v>
       </c>
       <c r="K30" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="L30" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="B31">
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="D31" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="E31" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="F31" t="s">
         <v>58</v>
       </c>
       <c r="G31" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="H31" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="I31" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="J31" t="s">
         <v>19</v>
       </c>
       <c r="K31" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="L31" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="B32">
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="D32" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="E32" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="F32" t="s">
         <v>58</v>
       </c>
       <c r="G32" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="H32" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="I32" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="J32" t="s">
         <v>19</v>
       </c>
       <c r="K32" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="L32" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="B33">
         <v>2</v>
       </c>
       <c r="C33" t="s">
+        <v>217</v>
+      </c>
+      <c r="D33" t="s">
+        <v>218</v>
+      </c>
+      <c r="E33" t="s">
+        <v>219</v>
+      </c>
+      <c r="F33" t="s">
+        <v>217</v>
+      </c>
+      <c r="G33" t="s">
+        <v>220</v>
+      </c>
+      <c r="H33" t="s">
+        <v>221</v>
+      </c>
+      <c r="I33" t="s">
+        <v>222</v>
+      </c>
+      <c r="J33" t="s">
+        <v>19</v>
+      </c>
+      <c r="K33" t="s">
         <v>223</v>
       </c>
-      <c r="D33" t="s">
-        <v>224</v>
-      </c>
-      <c r="E33" t="s">
-        <v>225</v>
-      </c>
-      <c r="F33" t="s">
-        <v>223</v>
-      </c>
-      <c r="G33" t="s">
-        <v>226</v>
-      </c>
-      <c r="H33" t="s">
-        <v>227</v>
-      </c>
-      <c r="I33" t="s">
-        <v>228</v>
-      </c>
-      <c r="J33" t="s">
-        <v>19</v>
-      </c>
-      <c r="K33" t="s">
-        <v>229</v>
-      </c>
       <c r="L33" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>